<commit_message>
Add json log and txt log
</commit_message>
<xml_diff>
--- a/employees.xlsx
+++ b/employees.xlsx
@@ -14,7 +14,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t>No</t>
+  </si>
   <si>
     <t>Name</t>
   </si>
@@ -351,27 +354,36 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
         <v>28</v>
       </c>
-      <c r="C2" t="s">
-        <v>4</v>
+      <c r="D2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3">
         <v>30</v>
       </c>
-      <c r="C3" t="s">
-        <v>6</v>
+      <c r="D3" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>